<commit_message>
update calendario e squadre
</commit_message>
<xml_diff>
--- a/risultati.xlsx
+++ b/risultati.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Utente\Documents\GitHub\12orebosaro\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3AC7103-5E63-4D39-8C19-C35B2B0D896C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84AEBB25-53A8-4AF9-9D07-77D2D11AF741}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1044" yWindow="2964" windowWidth="17280" windowHeight="8964" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3036" yWindow="3036" windowWidth="17280" windowHeight="8964" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Gironi" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="27">
   <si>
     <t>Girone</t>
   </si>
@@ -42,6 +42,66 @@
   </si>
   <si>
     <t>Esito (RigoriCasa/RigoriTrasferta)</t>
+  </si>
+  <si>
+    <t>D</t>
+  </si>
+  <si>
+    <t>All Blacks</t>
+  </si>
+  <si>
+    <t>Boldò Glimt</t>
+  </si>
+  <si>
+    <t>Coca Juniors</t>
+  </si>
+  <si>
+    <t>Piadineria La Salsiccia</t>
+  </si>
+  <si>
+    <t>B</t>
+  </si>
+  <si>
+    <t>Totani</t>
+  </si>
+  <si>
+    <t>Vecchie Glorie Rovigo Calcio</t>
+  </si>
+  <si>
+    <t>C</t>
+  </si>
+  <si>
+    <t>Leoni di Ricky</t>
+  </si>
+  <si>
+    <t>Pink 5ive</t>
+  </si>
+  <si>
+    <t>Barrio Boys</t>
+  </si>
+  <si>
+    <t>Cani</t>
+  </si>
+  <si>
+    <t>AS Bancatore</t>
+  </si>
+  <si>
+    <t>Beverton</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>Fatine FC</t>
+  </si>
+  <si>
+    <t>FC Internazionale Rovigo</t>
+  </si>
+  <si>
+    <t>MoViola Utd</t>
+  </si>
+  <si>
+    <t>Astolfi Impianti Elettrici</t>
   </si>
 </sst>
 </file>
@@ -387,8 +447,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="30.109375" customWidth="1"/>
+    <col min="3" max="3" width="30.44140625" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
@@ -408,6 +472,94 @@
       </c>
       <c r="F1" s="1" t="s">
         <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C6" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" t="s">
+        <v>20</v>
+      </c>
+      <c r="C7" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>22</v>
+      </c>
+      <c r="B8" t="s">
+        <v>23</v>
+      </c>
+      <c r="C8" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>22</v>
+      </c>
+      <c r="B9" t="s">
+        <v>25</v>
+      </c>
+      <c r="C9" t="s">
+        <v>26</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update Calendario e Gironi
</commit_message>
<xml_diff>
--- a/risultati.xlsx
+++ b/risultati.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Utente\Documents\GitHub\12orebosaro\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84AEBB25-53A8-4AF9-9D07-77D2D11AF741}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{239B469F-F040-4501-8B5D-A604FCA24B66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3036" yWindow="3036" windowWidth="17280" windowHeight="8964" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="28">
   <si>
     <t>Girone</t>
   </si>
@@ -102,6 +102,9 @@
   </si>
   <si>
     <t>Astolfi Impianti Elettrici</t>
+  </si>
+  <si>
+    <t>Vecchie Glorie Rovigo</t>
   </si>
 </sst>
 </file>
@@ -447,7 +450,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F25"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="30.109375" customWidth="1"/>
@@ -560,6 +563,182 @@
       </c>
       <c r="C9" t="s">
         <v>26</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>7</v>
+      </c>
+      <c r="B10" t="s">
+        <v>8</v>
+      </c>
+      <c r="C10" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>12</v>
+      </c>
+      <c r="B11" t="s">
+        <v>13</v>
+      </c>
+      <c r="C11" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B12" t="s">
+        <v>27</v>
+      </c>
+      <c r="C12" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>7</v>
+      </c>
+      <c r="B13" t="s">
+        <v>9</v>
+      </c>
+      <c r="C13" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>15</v>
+      </c>
+      <c r="B14" t="s">
+        <v>16</v>
+      </c>
+      <c r="C14" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>15</v>
+      </c>
+      <c r="B15" t="s">
+        <v>17</v>
+      </c>
+      <c r="C15" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>22</v>
+      </c>
+      <c r="B16" t="s">
+        <v>23</v>
+      </c>
+      <c r="C16" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>7</v>
+      </c>
+      <c r="B17" t="s">
+        <v>8</v>
+      </c>
+      <c r="C17" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>7</v>
+      </c>
+      <c r="B18" t="s">
+        <v>9</v>
+      </c>
+      <c r="C18" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>22</v>
+      </c>
+      <c r="B19" t="s">
+        <v>24</v>
+      </c>
+      <c r="C19" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>12</v>
+      </c>
+      <c r="B20" t="s">
+        <v>13</v>
+      </c>
+      <c r="C20" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>12</v>
+      </c>
+      <c r="B21" t="s">
+        <v>27</v>
+      </c>
+      <c r="C21" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>15</v>
+      </c>
+      <c r="B22" t="s">
+        <v>16</v>
+      </c>
+      <c r="C22" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>22</v>
+      </c>
+      <c r="B23" t="s">
+        <v>23</v>
+      </c>
+      <c r="C23" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>22</v>
+      </c>
+      <c r="B24" t="s">
+        <v>24</v>
+      </c>
+      <c r="C24" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>15</v>
+      </c>
+      <c r="B25" t="s">
+        <v>17</v>
+      </c>
+      <c r="C25" t="s">
+        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>